<commit_message>
All Refactorized: LLM as a players
</commit_message>
<xml_diff>
--- a/cards_dataset/EN/manual_configurations_5.xlsx
+++ b/cards_dataset/EN/manual_configurations_5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\!Master\Tesis\3 Mejorar codigo\Cards_Against_AI\cards_dataset\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2CDFA31-E323-496C-8072-6E7FC61C6875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA405D6C-F4B4-4187-90EA-2CFECECE9591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="200">
   <si>
     <t>black_id</t>
   </si>
@@ -614,6 +614,12 @@
   </si>
   <si>
     <t>W234</t>
+  </si>
+  <si>
+    <t>W041</t>
+  </si>
+  <si>
+    <t>W088</t>
   </si>
 </sst>
 </file>
@@ -1690,6 +1696,21 @@
       <c r="B32" t="s">
         <v>36</v>
       </c>
+      <c r="C32" t="s">
+        <v>181</v>
+      </c>
+      <c r="D32" t="s">
+        <v>198</v>
+      </c>
+      <c r="E32" t="s">
+        <v>120</v>
+      </c>
+      <c r="F32" t="s">
+        <v>138</v>
+      </c>
+      <c r="G32" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">

</xml_diff>